<commit_message>
fix typos spotted by Aleah
</commit_message>
<xml_diff>
--- a/data/aurignacian-periods.xlsx
+++ b/data/aurignacian-periods.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sophiecooper/Independent Research Study/SignBase/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bmarwick/Downloads/SignBase/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29507320-B411-8841-828B-EBA81E2C05D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F391AF0-6FC0-0C42-A290-7150D8DD7171}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="500" windowWidth="28040" windowHeight="16600" xr2:uid="{79486DA5-00F7-8844-88EA-52FFFB3FA67C}"/>
+    <workbookView xWindow="7620" yWindow="760" windowWidth="21180" windowHeight="16600" xr2:uid="{79486DA5-00F7-8844-88EA-52FFFB3FA67C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -92,10 +91,10 @@
     <t>GI 8 - 6</t>
   </si>
   <si>
-    <t>Preceeded by Greenland Stadial 12, ends with GI 11</t>
-  </si>
-  <si>
     <t>Begins with Henrich Stadial 4, ends with GI 8</t>
+  </si>
+  <si>
+    <t>Preceded by Greenland Stadial 12, ends with GI 11</t>
   </si>
 </sst>
 </file>
@@ -504,7 +503,7 @@
         <v>15</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="34" x14ac:dyDescent="0.2">
@@ -532,7 +531,7 @@
         <v>7</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="51" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
re-write with two phases
</commit_message>
<xml_diff>
--- a/data/aurignacian-periods.xlsx
+++ b/data/aurignacian-periods.xlsx
@@ -1,80 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11028"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bmarwick/Downloads/SignBase/data/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4424F35E-3300-1A4C-A3DA-0D68F088E4F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8580" yWindow="4740" windowWidth="18660" windowHeight="14180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
-  <si>
-    <t>Time Period Name</t>
-  </si>
-  <si>
-    <t>Dates (k cal BP)</t>
-  </si>
-  <si>
-    <t>Material Culture Markers</t>
-  </si>
-  <si>
-    <t>Environmental Context</t>
-  </si>
-  <si>
-    <t>Protoaurignacian</t>
-  </si>
-  <si>
-    <t>43 - 39.8</t>
-  </si>
-  <si>
-    <t>Spans Greenland Stadial 12 to GI 10 and 9</t>
-  </si>
-  <si>
-    <t>Early Aurignacian</t>
-  </si>
-  <si>
-    <t>39.8 - 37.8</t>
-  </si>
-  <si>
-    <t>Begins with Heinrich Stadial 4, ends with GI 8</t>
-  </si>
-  <si>
-    <t>Evolved/Late Aurignacian</t>
-  </si>
-  <si>
-    <t>37.8 - 32</t>
-  </si>
-  <si>
-    <t>GI 8 - 6</t>
-  </si>
-  <si>
-    <t>Blade and bladelet production now run as separate reduction sequences, with carinated and nosed end-scrapers systematically used as bladelet cores; thick blades with invasive, scalar Aurignacian retouch, sometimes waisted/strangled;  Dufour bladelets now include the smaller Roc-de-Combe subtype alongside Dufour; split-based antler/bone points (regionally variable)</t>
-  </si>
-  <si>
-    <t>Carinated/nosed-scraper bladelet-core technology intensifies further; busked (busqué) burins become numerous, later joined/replaced by the closely related Vachons-type burin; Dufour bladelets now dominated by the smaller, twisted Roc-de-Combe subtype, plus bipoint Font-Yves/Krems bladelets; split-based points disappear, replaced first by flattened lozenge-shaped bone/antler points (with the busked burins), then oval-sectioned lozenge points (with Vachons burins), and finally biconical points</t>
-  </si>
-  <si>
-    <t>Blades and bladelets produced within a single, continuous reduction sequence from the same unipolar/prismatic core, rather than from separate blade and bladelet cores; bladelets are the main target, large, straight-profiled, and turned into Dufour bladelets of the Dufour subtype via marginal direct, inverse or alternate retouch; bone/antler points are absent/very rare</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -111,16 +52,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -128,21 +63,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -180,7 +107,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -214,7 +141,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -249,10 +175,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -425,70 +350,74 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="21.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.33203125" customWidth="1"/>
-    <col min="3" max="3" width="64.33203125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="36" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Time Period Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Dates (k cal BP)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Material Culture Markers</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Environmental Context</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="80" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" t="s">
-        <v>6</v>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Aur-P1 (Proto/Early)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>43 - 37</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Blades and bladelets produced within a single, continuous reduction sequence from the same unipolar/prismatic core, rather than from separate blade and bladelet cores; bladelets are the main target, large, straight-profiled, and turned into Dufour bladelets of the Dufour subtype via marginal direct, inverse or alternate retouch; bone/antler points are absent/very rare Blade and bladelet production now run as separate reduction sequences, with carinated and nosed end-scrapers systematically used as bladelet cores; thick blades with invasive, scalar Aurignacian retouch, sometimes waisted/strangled;  Dufour bladelets now include the smaller Roc-de-Combe subtype alongside Dufour; split-based antler/bone points (regionally variable)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Spans Greenland Stadial 12 to GI 10 and 9 Begins with Heinrich Stadial 4, ends with GI 8</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="80" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="112" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" t="s">
-        <v>12</v>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Aur-P2 (Evolved/Late)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>37 - 32</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Carinated/nosed-scraper bladelet-core technology intensifies further; busked (busqué) burins become numerous, later joined/replaced by the closely related Vachons-type burin; Dufour bladelets now dominated by the smaller, twisted Roc-de-Combe subtype, plus bipoint Font-Yves/Krems bladelets; split-based points disappear, replaced first by flattened lozenge-shaped bone/antler points (with the busked burins), then oval-sectioned lozenge points (with Vachons burins), and finally biconical points</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>GI 8 - 6</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
layer-level Hohle Fels phase assignment; update results, supplements, and response
</commit_message>
<xml_diff>
--- a/data/aurignacian-periods.xlsx
+++ b/data/aurignacian-periods.xlsx
@@ -1,21 +1,68 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11028"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bmarwick/Downloads/SignBase/data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{984D0BB6-6592-0C4F-AAB1-38ACFC28BB01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="240" yWindow="760" windowWidth="16100" windowHeight="16820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+  <si>
+    <t>Time Period Name</t>
+  </si>
+  <si>
+    <t>Dates (k cal BP)</t>
+  </si>
+  <si>
+    <t>Material Culture Markers</t>
+  </si>
+  <si>
+    <t>Environmental Context</t>
+  </si>
+  <si>
+    <t>Aur-P1 (Proto/Early)</t>
+  </si>
+  <si>
+    <t>43 - 37</t>
+  </si>
+  <si>
+    <t>Aur-P2 (Evolved/Late)</t>
+  </si>
+  <si>
+    <t>37 - 32</t>
+  </si>
+  <si>
+    <t>GI 8 - 6</t>
+  </si>
+  <si>
+    <t>Starts at Greenland Stadial 12, ends at Greenland  Interstadial 8</t>
+  </si>
+  <si>
+    <t>Blades and bladelets intially produced within a single, continuous reduction sequence from the same unipolar/prismatic core, rather than from separate blade and bladelet cores; bladelets are the main target, large, straight-profiled, and turned into Dufour bladelets of the Dufour subtype via marginal direct, inverse or alternate retouch; bone/antler points are initially very rare, then regionally variable. Blade and bladelet production later run as separate reduction sequences, with carinated and nosed end-scrapers systematically used as bladelet cores; thick blades with invasive, scalar Aurignacian retouch, sometimes waisted/strangled;  Dufour bladelets later include the smaller Roc-de-Combe subtype alongside Dufour.</t>
+  </si>
+  <si>
+    <t>Carinated/nosed-scraper bladelet-core technology intensifies further; busked (busqué) burins become numerous, later joined/replaced by the closely related Vachons-type burin; Dufour bladelets now dominated by the smaller, twisted Roc-de-Combe subtype; split-based points become rare, replaced first by flattened lozenge-shaped bone/antler points (with the busked burins), then oval-sectioned lozenge points (with Vachons burins), and finally biconical points</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -63,13 +110,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -107,7 +162,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -141,6 +196,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -175,9 +231,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -350,74 +407,55 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="26.1640625" customWidth="1"/>
+    <col min="2" max="2" width="21.5" customWidth="1"/>
+    <col min="3" max="3" width="30.1640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Time Period Name</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Dates (k cal BP)</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Material Culture Markers</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Environmental Context</t>
-        </is>
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Aur-P1 (Proto/Early)</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>43 - 37</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Blades and bladelets produced within a single, continuous reduction sequence from the same unipolar/prismatic core, rather than from separate blade and bladelet cores; bladelets are the main target, large, straight-profiled, and turned into Dufour bladelets of the Dufour subtype via marginal direct, inverse or alternate retouch; bone/antler points are absent/very rare Blade and bladelet production now run as separate reduction sequences, with carinated and nosed end-scrapers systematically used as bladelet cores; thick blades with invasive, scalar Aurignacian retouch, sometimes waisted/strangled;  Dufour bladelets now include the smaller Roc-de-Combe subtype alongside Dufour; split-based antler/bone points (regionally variable)</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Spans Greenland Stadial 12 to GI 10 and 9 Begins with Heinrich Stadial 4, ends with GI 8</t>
-        </is>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Aur-P2 (Evolved/Late)</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>37 - 32</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Carinated/nosed-scraper bladelet-core technology intensifies further; busked (busqué) burins become numerous, later joined/replaced by the closely related Vachons-type burin; Dufour bladelets now dominated by the smaller, twisted Roc-de-Combe subtype, plus bipoint Font-Yves/Krems bladelets; split-based points disappear, replaced first by flattened lozenge-shaped bone/antler points (with the busked burins), then oval-sectioned lozenge points (with Vachons burins), and finally biconical points</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>GI 8 - 6</t>
-        </is>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refresh reply to reviewers
</commit_message>
<xml_diff>
--- a/data/aurignacian-periods.xlsx
+++ b/data/aurignacian-periods.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bmarwick/Downloads/SignBase/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{252DCB80-4B2B-F243-BC35-62070BC829E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{780E6BCB-1032-2645-BA07-4C81C492B290}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="760" windowWidth="16100" windowHeight="16820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -55,7 +55,7 @@
     <t>Dates (ka cal BP)</t>
   </si>
   <si>
-    <t>Blades and bladelets initially produced within a single, continuous reduction sequence from the same unipolar/prismatic core, rather than from separate blade and bladelet cores; bladelets are the main target, large, straight-profiled, and turned into Dufour bladelets of the Dufour subtype via marginal direct, inverse or alternate retouch; bone/antler points are initially very rare, then regionally variable. Blade and bladelet production later run as separate reduction sequences, with carinated and nosed end-scrapers systematically used as bladelet cores; thick blades with invasive, scalar Aurignacian retouch, sometimes waisted/strangled;  Dufour bladelets later include the smaller Roc-de-Combe subtype alongside Dufour.</t>
+    <t>Blades and bladelets initially produced within a single, continuous reduction sequence from the same unipolar/prismatic core, rather than from separate blade and bladelet cores; bladelets are the main target, large, straight-profiled, and turned into Dufour bladelets of the Dufour subtype via marginal direct, inverse or alternate retouch; split-based bone/antler points are initially very rare, then regionally variable. Blade and bladelet production later run as separate reduction sequences, with carinated and nosed end-scrapers systematically used as bladelet cores; thick blades with invasive, scalar Aurignacian retouch, sometimes waisted/strangled;  Dufour bladelets later include the smaller Roc-de-Combe subtype alongside Dufour.</t>
   </si>
 </sst>
 </file>

</xml_diff>